<commit_message>
Update details on 8june
</commit_message>
<xml_diff>
--- a/public/Students_Final.xlsx
+++ b/public/Students_Final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/swapnilbaranwal/Desktop/Important documents/friends-library_bareilly/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6B163B7-442A-0D47-B707-78715544DC33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D2CAEC-207D-EF42-B77A-020C1A7EAF3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="57">
   <si>
     <t>S.No.</t>
   </si>
@@ -173,6 +173,24 @@
   </si>
   <si>
     <t>Naveen</t>
+  </si>
+  <si>
+    <t>Manasvi</t>
+  </si>
+  <si>
+    <t>Manas</t>
+  </si>
+  <si>
+    <t>Anuj</t>
+  </si>
+  <si>
+    <t>Unpaid</t>
+  </si>
+  <si>
+    <t>Vikash</t>
+  </si>
+  <si>
+    <t>Vipin</t>
   </si>
 </sst>
 </file>
@@ -595,7 +613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S32"/>
+  <dimension ref="A1:S37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -1147,7 +1165,7 @@
         <v>32</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="D13" s="9">
         <v>46121</v>
@@ -1155,9 +1173,7 @@
       <c r="E13" s="10">
         <v>700</v>
       </c>
-      <c r="F13" s="7">
-        <v>35</v>
-      </c>
+      <c r="F13" s="7"/>
       <c r="G13" s="6" t="s">
         <v>21</v>
       </c>
@@ -1173,7 +1189,9 @@
       <c r="K13" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="L13" s="7"/>
+      <c r="L13" s="6" t="s">
+        <v>21</v>
+      </c>
       <c r="M13" s="7"/>
       <c r="N13" s="7"/>
       <c r="O13" s="7"/>
@@ -1216,7 +1234,9 @@
       <c r="K14" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="L14" s="2"/>
+      <c r="L14" s="2" t="s">
+        <v>47</v>
+      </c>
       <c r="M14" s="2"/>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -1544,9 +1564,7 @@
       <c r="E22" s="5">
         <v>700</v>
       </c>
-      <c r="F22" s="2">
-        <v>42</v>
-      </c>
+      <c r="F22" s="2"/>
       <c r="G22" s="6" t="s">
         <v>21</v>
       </c>
@@ -1753,7 +1771,7 @@
         <v>46</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="D27" s="9">
         <v>46148</v>
@@ -1761,9 +1779,7 @@
       <c r="E27" s="10">
         <v>700</v>
       </c>
-      <c r="F27" s="7">
-        <v>24</v>
-      </c>
+      <c r="F27" s="7"/>
       <c r="G27" s="6" t="s">
         <v>21</v>
       </c>
@@ -1779,7 +1795,9 @@
       <c r="K27" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="L27" s="7"/>
+      <c r="L27" s="6" t="s">
+        <v>21</v>
+      </c>
       <c r="M27" s="7"/>
       <c r="N27" s="7"/>
       <c r="O27" s="7"/>
@@ -2009,9 +2027,234 @@
       <c r="R32" s="2"/>
       <c r="S32" s="2"/>
     </row>
+    <row r="33" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="2">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="4">
+        <v>46175</v>
+      </c>
+      <c r="E33" s="5">
+        <v>700</v>
+      </c>
+      <c r="F33" s="2">
+        <v>15</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I33" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L33" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="M33" s="2"/>
+      <c r="N33" s="2"/>
+      <c r="O33" s="2"/>
+      <c r="P33" s="2"/>
+      <c r="Q33" s="2"/>
+      <c r="R33" s="2"/>
+      <c r="S33" s="2"/>
+    </row>
+    <row r="34" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="2">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D34" s="4">
+        <v>46180</v>
+      </c>
+      <c r="E34" s="5">
+        <v>700</v>
+      </c>
+      <c r="F34" s="2">
+        <v>12</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I34" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="M34" s="2"/>
+      <c r="N34" s="2"/>
+      <c r="O34" s="2"/>
+      <c r="P34" s="2"/>
+      <c r="Q34" s="2"/>
+      <c r="R34" s="2"/>
+      <c r="S34" s="2"/>
+    </row>
+    <row r="35" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="2">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D35" s="4">
+        <v>46181</v>
+      </c>
+      <c r="E35" s="5">
+        <v>700</v>
+      </c>
+      <c r="F35" s="2">
+        <v>11</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L35" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="M35" s="2"/>
+      <c r="N35" s="2"/>
+      <c r="O35" s="2"/>
+      <c r="P35" s="2"/>
+      <c r="Q35" s="2"/>
+      <c r="R35" s="2"/>
+      <c r="S35" s="2"/>
+    </row>
+    <row r="36" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="2">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D36" s="4">
+        <v>46178</v>
+      </c>
+      <c r="E36" s="5">
+        <v>700</v>
+      </c>
+      <c r="F36" s="2">
+        <v>41</v>
+      </c>
+      <c r="G36" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J36" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K36" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="M36" s="2"/>
+      <c r="N36" s="2"/>
+      <c r="O36" s="2"/>
+      <c r="P36" s="2"/>
+      <c r="Q36" s="2"/>
+      <c r="R36" s="2"/>
+      <c r="S36" s="2"/>
+    </row>
+    <row r="37" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="2">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D37" s="4">
+        <v>46178</v>
+      </c>
+      <c r="E37" s="5">
+        <v>700</v>
+      </c>
+      <c r="F37" s="2">
+        <v>42</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J37" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L37" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="M37" s="2"/>
+      <c r="N37" s="2"/>
+      <c r="O37" s="2"/>
+      <c r="P37" s="2"/>
+      <c r="Q37" s="2"/>
+      <c r="R37" s="2"/>
+      <c r="S37" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="K10:K29 I26 J2 I4:J4 J6 J9:J11 J13:J14 J17 J19 J21:J26 G10:I10 K2:K8 M2:S32 L23:L32 L2:L20" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="K10:K29 I26 J2 I4:J4 J6 J9:J11 J13:J14 J17 J19 J21:J26 G10:I10 K2:K8 M2:S37 L14:L20 L2:L12 L23:L26 L28:L37" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Paid,Unpaid"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>